<commit_message>
Fase 3: test por bloques con avance guardado y reanudación
- views/test.py: preguntas por bloque (10), barra de avance, opciones de 44 px,
  instrucciones por test (hoja info) y pantalla final. Todas obligatorias.
- modules/avance.py: posición del alumno, guardado por bloque, cierre de test y alumno,
  detección de cambio de versión del test.
- Opción SE como NULL; SupabaseRepo con progreso y respuestas (upsert idempotente).
- 92 pruebas; verificado en celular emulado y contra Supabase (alumno temporal borrado).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/tests/1_test_big_five.xlsx
+++ b/config/tests/1_test_big_five.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -440,6 +440,18 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>Big Five (OCEAN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>instrucciones</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Evalúa cada afirmación indicando qué tan identificado/a te sientes en tu desempeño académico y profesional.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fase 4: calificación, resultados y reportes PDF/Excel del alumno
- modules/scoring.py: puntajes, SE como dato faltante, afinidades derivadas, ranking con
  desempate y empate técnico. Verificado contra las calculadoras de Excel (253 casos).
- Cargador: hojas opcionales niveles y afinidad; version_test solo depende de preguntas/escala.
- modules/reports.py: PDF y Excel individuales, vista conjunta y radar; sin fórmulas inyectables.
- Pantalla final: el alumno ve sus resultados y descarga PDF y Excel.
- Nombres deben empezar con letra; resultados.especialidad_principal admite NULL.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/tests/1_test_big_five.xlsx
+++ b/config/tests/1_test_big_five.xlsx
@@ -11,6 +11,8 @@
     <sheet name="especialidades" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="preguntas" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="escala" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="niveles" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="afinidad" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1306,4 +1308,271 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ambito</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>minimo</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>etiqueta</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>categoria</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>categoria</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>categoria</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Área de Desarrollo</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>afinidad</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Alta Afinidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>afinidad</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Afinidad Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>afinidad</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Desarrollo Requerido</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>codigo</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>nombre</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>componentes</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>descripcion</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MKT</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mercadotecnia</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>APERTURA+EXTRAVERSION</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Creatividad, visión de mercado, dinamismo social y comunicación persuasiva.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Capital Humano</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>AMABILIDAD+EXTRAVERSION</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Gestión del talento, empatía organizacional, mediación y liderazgo de equipos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AF</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Administración Financiera</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>RESPONSABILIDAD+ESTABILIDAD</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Rigor cuantitativo, control de riesgos, disciplina y toma de decisiones bajo presión.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NI</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Negocios Internacionales</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>APERTURA+ESTABILIDAD+EXTRAVERSION</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Inteligencia cultural, adaptabilidad global, resiliencia y capacidad de negociación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>EMP</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Emprendimiento</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>APERTURA+RESPONSABILIDAD+ESTABILIDAD</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Visión de oportunidad, autodisciplina ejecutiva, resiliencia y tolerancia al riesgo.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>